<commit_message>
frontend: fix bugs and redirects, seo
</commit_message>
<xml_diff>
--- a/addact/public/redirects.xlsx
+++ b/addact/public/redirects.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Addact-Revamp\addact\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\Addact-Revamp\addact\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C672DA5-AF58-4C0F-8C4D-C00EAFE09370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D088DA5C-078C-4D7F-A278-20525E1ED177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5F6600C6-C08A-47D2-B3C8-F7A43562057B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="654">
   <si>
     <t>source</t>
   </si>
@@ -1919,9 +1919,6 @@
     <t>/blogs/increase-customer-loyalty-and-trust-using-sitecore-cdp</t>
   </si>
   <si>
-    <t>/project-cost-estimator</t>
-  </si>
-  <si>
     <t>/role-of-sitecore-cdp-customer-experience-management</t>
   </si>
   <si>
@@ -1929,6 +1926,78 @@
   </si>
   <si>
     <t>/blogs/how-to-migrate-from-a-legacy-cms-to-sitecore-challenges-and-solutions</t>
+  </si>
+  <si>
+    <t>/development-design/cms-development/sitecore</t>
+  </si>
+  <si>
+    <t>/umbraco-cms-development</t>
+  </si>
+  <si>
+    <t>/development-design/cms-development/umbraco</t>
+  </si>
+  <si>
+    <t>/strapi-cms-development</t>
+  </si>
+  <si>
+    <t>/development-design/cms-development/strapi</t>
+  </si>
+  <si>
+    <t>/kentico-cms-development</t>
+  </si>
+  <si>
+    <t>/development-design/cms-development/kentico</t>
+  </si>
+  <si>
+    <t>/contentful-cms-development</t>
+  </si>
+  <si>
+    <t>/development-design/cms-development/contentful</t>
+  </si>
+  <si>
+    <t>/contentstack-cms-development</t>
+  </si>
+  <si>
+    <t>/development-design/cms-development/contentstack</t>
+  </si>
+  <si>
+    <t>/development-design/cms-development/sitecore/support-and-maintenance</t>
+  </si>
+  <si>
+    <t>/development-design/cms-development/sitecore/consulting-services</t>
+  </si>
+  <si>
+    <t>/development-design/cms-development/sitecore/sitecore-ai</t>
+  </si>
+  <si>
+    <t>/development-design/cms-development/sitecore/platform-integrations</t>
+  </si>
+  <si>
+    <t>/development-design/cms-development/sitecore/audit-service</t>
+  </si>
+  <si>
+    <t>/development-design/cms-development/sitecore/platform-upgrade</t>
+  </si>
+  <si>
+    <t>/hire-experts/sitecore-developer</t>
+  </si>
+  <si>
+    <t>/umbraco-cms-development/hire-umbraco-developer</t>
+  </si>
+  <si>
+    <t>/hire-experts/umbraco-developer</t>
+  </si>
+  <si>
+    <t>/strapi-cms-development/hire-strapi-developer</t>
+  </si>
+  <si>
+    <t>/hire-experts/strapi-developer</t>
+  </si>
+  <si>
+    <t>/kentico-cms-development/hire-kentico-developer</t>
+  </si>
+  <si>
+    <t>/hire-experts/kentico-developer</t>
   </si>
 </sst>
 </file>
@@ -2358,15 +2427,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C59FA00F-2D8F-4BC7-B234-D60C0BA408AE}">
-  <dimension ref="A1:C331"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C346"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="107.44140625" customWidth="1"/>
     <col min="2" max="2" width="83.109375" customWidth="1"/>
     <col min="3" max="3" width="14.21875" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" s="1">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2377,7 +2446,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
@@ -2388,7 +2457,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>16</v>
       </c>
@@ -2399,7 +2468,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>18</v>
       </c>
@@ -2410,7 +2479,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>20</v>
       </c>
@@ -2421,7 +2490,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>22</v>
       </c>
@@ -2432,7 +2501,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>24</v>
       </c>
@@ -2443,7 +2512,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>26</v>
       </c>
@@ -2454,7 +2523,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>28</v>
       </c>
@@ -2465,7 +2534,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>30</v>
       </c>
@@ -2476,7 +2545,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>32</v>
       </c>
@@ -2487,18 +2556,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>34</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>35</v>
       </c>
@@ -2509,7 +2578,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>37</v>
       </c>
@@ -2520,7 +2589,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>39</v>
       </c>
@@ -2531,7 +2600,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
         <v>41</v>
       </c>
@@ -2542,7 +2611,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
         <v>43</v>
       </c>
@@ -2553,7 +2622,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>45</v>
       </c>
@@ -2564,7 +2633,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>47</v>
       </c>
@@ -2575,7 +2644,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>49</v>
       </c>
@@ -2586,7 +2655,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
         <v>51</v>
       </c>
@@ -2597,7 +2666,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
         <v>53</v>
       </c>
@@ -2608,7 +2677,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
         <v>55</v>
       </c>
@@ -2619,7 +2688,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
         <v>57</v>
       </c>
@@ -2630,7 +2699,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
         <v>59</v>
       </c>
@@ -2641,7 +2710,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
         <v>61</v>
       </c>
@@ -2652,7 +2721,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
         <v>63</v>
       </c>
@@ -2663,7 +2732,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
         <v>65</v>
       </c>
@@ -2674,7 +2743,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
         <v>67</v>
       </c>
@@ -2685,7 +2754,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>69</v>
       </c>
@@ -2696,7 +2765,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>71</v>
       </c>
@@ -2707,7 +2776,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>73</v>
       </c>
@@ -2718,7 +2787,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
         <v>75</v>
       </c>
@@ -2729,7 +2798,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
         <v>77</v>
       </c>
@@ -2740,7 +2809,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
         <v>79</v>
       </c>
@@ -2751,7 +2820,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="8" t="s">
         <v>81</v>
       </c>
@@ -2762,7 +2831,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="8" t="s">
         <v>83</v>
       </c>
@@ -2773,7 +2842,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="8" t="s">
         <v>85</v>
       </c>
@@ -2784,7 +2853,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="8" t="s">
         <v>87</v>
       </c>
@@ -2795,7 +2864,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="8" t="s">
         <v>89</v>
       </c>
@@ -2806,7 +2875,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="8" t="s">
         <v>91</v>
       </c>
@@ -2817,7 +2886,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="8" t="s">
         <v>93</v>
       </c>
@@ -2828,7 +2897,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" ht="27">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="9" t="s">
         <v>95</v>
       </c>
@@ -2839,7 +2908,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="8" t="s">
         <v>97</v>
       </c>
@@ -2850,7 +2919,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="8" t="s">
         <v>99</v>
       </c>
@@ -2861,7 +2930,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="8" t="s">
         <v>101</v>
       </c>
@@ -2872,7 +2941,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="8" t="s">
         <v>103</v>
       </c>
@@ -2883,7 +2952,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="8" t="s">
         <v>105</v>
       </c>
@@ -2894,7 +2963,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="8" t="s">
         <v>107</v>
       </c>
@@ -2905,7 +2974,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="8" t="s">
         <v>109</v>
       </c>
@@ -2916,7 +2985,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="8" t="s">
         <v>111</v>
       </c>
@@ -2927,7 +2996,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="8" t="s">
         <v>113</v>
       </c>
@@ -2938,7 +3007,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="8" t="s">
         <v>115</v>
       </c>
@@ -2949,7 +3018,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="8" t="s">
         <v>117</v>
       </c>
@@ -2960,7 +3029,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="8" t="s">
         <v>119</v>
       </c>
@@ -2971,7 +3040,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="8" t="s">
         <v>121</v>
       </c>
@@ -2982,7 +3051,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="8" t="s">
         <v>123</v>
       </c>
@@ -2993,7 +3062,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" s="8" t="s">
         <v>125</v>
       </c>
@@ -3004,7 +3073,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" s="8" t="s">
         <v>127</v>
       </c>
@@ -3015,7 +3084,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" s="8" t="s">
         <v>129</v>
       </c>
@@ -3026,7 +3095,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" s="8" t="s">
         <v>131</v>
       </c>
@@ -3037,7 +3106,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" s="8" t="s">
         <v>133</v>
       </c>
@@ -3048,7 +3117,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" s="8" t="s">
         <v>135</v>
       </c>
@@ -3059,7 +3128,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="64" ht="27">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" s="9" t="s">
         <v>137</v>
       </c>
@@ -3070,7 +3139,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" s="8" t="s">
         <v>139</v>
       </c>
@@ -3081,7 +3150,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" s="8" t="s">
         <v>141</v>
       </c>
@@ -3092,7 +3161,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" s="8" t="s">
         <v>143</v>
       </c>
@@ -3103,7 +3172,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" s="8" t="s">
         <v>145</v>
       </c>
@@ -3114,7 +3183,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" s="8" t="s">
         <v>147</v>
       </c>
@@ -3125,7 +3194,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" s="8" t="s">
         <v>149</v>
       </c>
@@ -3136,7 +3205,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="71" ht="27">
+    <row r="71" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A71" s="9" t="s">
         <v>151</v>
       </c>
@@ -3147,7 +3216,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" ht="27">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" s="9" t="s">
         <v>153</v>
       </c>
@@ -3158,7 +3227,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" s="8" t="s">
         <v>155</v>
       </c>
@@ -3169,7 +3238,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" s="8" t="s">
         <v>157</v>
       </c>
@@ -3180,7 +3249,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" ht="27">
+    <row r="75" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A75" s="9" t="s">
         <v>159</v>
       </c>
@@ -3191,7 +3260,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" s="8" t="s">
         <v>161</v>
       </c>
@@ -3202,7 +3271,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" s="8" t="s">
         <v>163</v>
       </c>
@@ -3213,7 +3282,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" s="8" t="s">
         <v>165</v>
       </c>
@@ -3224,7 +3293,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" s="8" t="s">
         <v>167</v>
       </c>
@@ -3235,7 +3304,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" s="8" t="s">
         <v>169</v>
       </c>
@@ -3246,7 +3315,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" s="8" t="s">
         <v>171</v>
       </c>
@@ -3257,7 +3326,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" s="8" t="s">
         <v>173</v>
       </c>
@@ -3268,7 +3337,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" s="8" t="s">
         <v>175</v>
       </c>
@@ -3279,7 +3348,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" s="8" t="s">
         <v>177</v>
       </c>
@@ -3290,7 +3359,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" s="8" t="s">
         <v>179</v>
       </c>
@@ -3301,7 +3370,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" s="8" t="s">
         <v>181</v>
       </c>
@@ -3312,7 +3381,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" s="8" t="s">
         <v>183</v>
       </c>
@@ -3323,7 +3392,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" s="8" t="s">
         <v>185</v>
       </c>
@@ -3334,7 +3403,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" s="8" t="s">
         <v>187</v>
       </c>
@@ -3345,7 +3414,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" s="8" t="s">
         <v>189</v>
       </c>
@@ -3356,7 +3425,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" s="8" t="s">
         <v>191</v>
       </c>
@@ -3367,7 +3436,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" s="8" t="s">
         <v>193</v>
       </c>
@@ -3378,7 +3447,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" s="8" t="s">
         <v>195</v>
       </c>
@@ -3389,7 +3458,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" s="8" t="s">
         <v>197</v>
       </c>
@@ -3400,7 +3469,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="95" ht="27">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" s="9" t="s">
         <v>199</v>
       </c>
@@ -3411,7 +3480,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" s="8" t="s">
         <v>201</v>
       </c>
@@ -3422,7 +3491,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" s="8" t="s">
         <v>203</v>
       </c>
@@ -3433,7 +3502,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" s="8" t="s">
         <v>205</v>
       </c>
@@ -3444,7 +3513,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="99" ht="27">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" s="9" t="s">
         <v>207</v>
       </c>
@@ -3455,7 +3524,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" s="8" t="s">
         <v>209</v>
       </c>
@@ -3466,7 +3535,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" s="8" t="s">
         <v>211</v>
       </c>
@@ -3477,7 +3546,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" s="8" t="s">
         <v>213</v>
       </c>
@@ -3488,7 +3557,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="103">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" s="8" t="s">
         <v>215</v>
       </c>
@@ -3499,7 +3568,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A104" s="8" t="s">
         <v>217</v>
       </c>
@@ -3510,7 +3579,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" s="8" t="s">
         <v>219</v>
       </c>
@@ -3521,7 +3590,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="106">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A106" s="8" t="s">
         <v>221</v>
       </c>
@@ -3532,7 +3601,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A107" s="8" t="s">
         <v>223</v>
       </c>
@@ -3543,7 +3612,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A108" s="8" t="s">
         <v>225</v>
       </c>
@@ -3554,7 +3623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="109">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A109" s="8" t="s">
         <v>227</v>
       </c>
@@ -3565,7 +3634,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="110">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A110" s="8" t="s">
         <v>229</v>
       </c>
@@ -3576,7 +3645,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="111">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A111" s="8" t="s">
         <v>231</v>
       </c>
@@ -3587,7 +3656,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="112">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A112" s="8" t="s">
         <v>233</v>
       </c>
@@ -3598,7 +3667,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="113">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" s="8" t="s">
         <v>235</v>
       </c>
@@ -3609,7 +3678,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="114">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A114" s="8" t="s">
         <v>237</v>
       </c>
@@ -3620,7 +3689,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="115">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A115" s="8" t="s">
         <v>239</v>
       </c>
@@ -3631,7 +3700,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="116">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A116" s="8" t="s">
         <v>241</v>
       </c>
@@ -3642,7 +3711,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="117" ht="27">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A117" s="9" t="s">
         <v>243</v>
       </c>
@@ -3653,7 +3722,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="118">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A118" s="8" t="s">
         <v>245</v>
       </c>
@@ -3664,7 +3733,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="119">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A119" s="8" t="s">
         <v>247</v>
       </c>
@@ -3675,7 +3744,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="120">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A120" s="8" t="s">
         <v>249</v>
       </c>
@@ -3686,7 +3755,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="121">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A121" s="8" t="s">
         <v>251</v>
       </c>
@@ -3697,7 +3766,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="122" ht="27">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A122" s="9" t="s">
         <v>253</v>
       </c>
@@ -3708,7 +3777,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="123">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A123" s="8" t="s">
         <v>255</v>
       </c>
@@ -3719,7 +3788,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="124">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A124" s="8" t="s">
         <v>257</v>
       </c>
@@ -3730,7 +3799,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="125">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A125" s="8" t="s">
         <v>259</v>
       </c>
@@ -3741,7 +3810,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="126">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A126" s="8" t="s">
         <v>261</v>
       </c>
@@ -3752,7 +3821,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="127">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A127" s="8" t="s">
         <v>263</v>
       </c>
@@ -3763,7 +3832,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="128">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A128" s="8" t="s">
         <v>265</v>
       </c>
@@ -3774,7 +3843,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="129">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A129" s="8" t="s">
         <v>267</v>
       </c>
@@ -3785,7 +3854,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="130">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A130" s="8" t="s">
         <v>269</v>
       </c>
@@ -3796,7 +3865,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="131">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A131" s="8" t="s">
         <v>271</v>
       </c>
@@ -3807,7 +3876,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="132">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A132" s="8" t="s">
         <v>273</v>
       </c>
@@ -3818,7 +3887,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="133">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A133" s="8" t="s">
         <v>275</v>
       </c>
@@ -3829,7 +3898,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="134">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A134" s="8" t="s">
         <v>277</v>
       </c>
@@ -3840,7 +3909,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="135">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A135" s="8" t="s">
         <v>279</v>
       </c>
@@ -3851,7 +3920,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="136">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A136" s="8" t="s">
         <v>281</v>
       </c>
@@ -3862,7 +3931,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="137">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A137" s="8" t="s">
         <v>283</v>
       </c>
@@ -3873,7 +3942,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="138">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A138" s="8" t="s">
         <v>285</v>
       </c>
@@ -3884,7 +3953,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="139" ht="27">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A139" s="9" t="s">
         <v>287</v>
       </c>
@@ -3895,7 +3964,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="140">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A140" s="8" t="s">
         <v>289</v>
       </c>
@@ -3906,7 +3975,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="141">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A141" s="8" t="s">
         <v>291</v>
       </c>
@@ -3917,7 +3986,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="142">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A142" s="8" t="s">
         <v>293</v>
       </c>
@@ -3928,7 +3997,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="143">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A143" s="8" t="s">
         <v>295</v>
       </c>
@@ -3939,7 +4008,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="144">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A144" s="8" t="s">
         <v>297</v>
       </c>
@@ -3950,7 +4019,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="145">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A145" s="8" t="s">
         <v>299</v>
       </c>
@@ -3961,7 +4030,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="146">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A146" s="8" t="s">
         <v>301</v>
       </c>
@@ -3972,7 +4041,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="147">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A147" s="8" t="s">
         <v>303</v>
       </c>
@@ -3983,7 +4052,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="148">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A148" s="8" t="s">
         <v>305</v>
       </c>
@@ -3994,7 +4063,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="149">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A149" s="8" t="s">
         <v>307</v>
       </c>
@@ -4005,7 +4074,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="150">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A150" s="8" t="s">
         <v>309</v>
       </c>
@@ -4016,7 +4085,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="151">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A151" s="8" t="s">
         <v>311</v>
       </c>
@@ -4027,7 +4096,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="152">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A152" s="8" t="s">
         <v>313</v>
       </c>
@@ -4038,7 +4107,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="153">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A153" s="8" t="s">
         <v>315</v>
       </c>
@@ -4049,7 +4118,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="154">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A154" s="8" t="s">
         <v>317</v>
       </c>
@@ -4060,7 +4129,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="155">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A155" s="8" t="s">
         <v>319</v>
       </c>
@@ -4071,7 +4140,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="156">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A156" s="8" t="s">
         <v>321</v>
       </c>
@@ -4082,7 +4151,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="157">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A157" s="8" t="s">
         <v>323</v>
       </c>
@@ -4093,7 +4162,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="158">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A158" s="8" t="s">
         <v>325</v>
       </c>
@@ -4104,7 +4173,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="159">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A159" s="8" t="s">
         <v>327</v>
       </c>
@@ -4115,7 +4184,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="160">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A160" s="8" t="s">
         <v>329</v>
       </c>
@@ -4126,7 +4195,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="161">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A161" s="8" t="s">
         <v>331</v>
       </c>
@@ -4137,7 +4206,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="162">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A162" s="8" t="s">
         <v>333</v>
       </c>
@@ -4148,7 +4217,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="163">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A163" s="8" t="s">
         <v>335</v>
       </c>
@@ -4159,7 +4228,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="164">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A164" s="8" t="s">
         <v>337</v>
       </c>
@@ -4170,7 +4239,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="165">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A165" s="8" t="s">
         <v>339</v>
       </c>
@@ -4181,7 +4250,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="166">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A166" s="8" t="s">
         <v>341</v>
       </c>
@@ -4192,7 +4261,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="167">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A167" s="8" t="s">
         <v>343</v>
       </c>
@@ -4203,7 +4272,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="168">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A168" s="8" t="s">
         <v>345</v>
       </c>
@@ -4214,7 +4283,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="169">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A169" s="8" t="s">
         <v>347</v>
       </c>
@@ -4225,7 +4294,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="170">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A170" s="8" t="s">
         <v>349</v>
       </c>
@@ -4236,7 +4305,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="171">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A171" s="8" t="s">
         <v>351</v>
       </c>
@@ -4247,7 +4316,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="172">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A172" s="8" t="s">
         <v>353</v>
       </c>
@@ -4258,7 +4327,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="173">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A173" s="8" t="s">
         <v>355</v>
       </c>
@@ -4269,7 +4338,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="174">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A174" s="8" t="s">
         <v>357</v>
       </c>
@@ -4280,7 +4349,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="175">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A175" s="8" t="s">
         <v>359</v>
       </c>
@@ -4291,7 +4360,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="176">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A176" s="8" t="s">
         <v>361</v>
       </c>
@@ -4302,7 +4371,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="177">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A177" s="8" t="s">
         <v>363</v>
       </c>
@@ -4313,7 +4382,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="178">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A178" s="8" t="s">
         <v>365</v>
       </c>
@@ -4324,7 +4393,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="179">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A179" s="8" t="s">
         <v>367</v>
       </c>
@@ -4335,7 +4404,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="180">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A180" s="8" t="s">
         <v>369</v>
       </c>
@@ -4346,7 +4415,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="181">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A181" s="8" t="s">
         <v>371</v>
       </c>
@@ -4357,7 +4426,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="182">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A182" s="8" t="s">
         <v>373</v>
       </c>
@@ -4368,7 +4437,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="183" ht="42">
+    <row r="183" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A183" s="9" t="s">
         <v>375</v>
       </c>
@@ -4379,7 +4448,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="184">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A184" s="8" t="s">
         <v>377</v>
       </c>
@@ -4390,7 +4459,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="185">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A185" s="8" t="s">
         <v>379</v>
       </c>
@@ -4401,7 +4470,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="186">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A186" s="8" t="s">
         <v>381</v>
       </c>
@@ -4412,7 +4481,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="187">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A187" s="8" t="s">
         <v>383</v>
       </c>
@@ -4423,7 +4492,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="188">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A188" s="8" t="s">
         <v>385</v>
       </c>
@@ -4434,7 +4503,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="189">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A189" s="8" t="s">
         <v>387</v>
       </c>
@@ -4445,7 +4514,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="190">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A190" s="8" t="s">
         <v>389</v>
       </c>
@@ -4456,7 +4525,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="191">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A191" s="8" t="s">
         <v>391</v>
       </c>
@@ -4467,7 +4536,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="192">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A192" s="8" t="s">
         <v>393</v>
       </c>
@@ -4478,7 +4547,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="193">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A193" s="8" t="s">
         <v>395</v>
       </c>
@@ -4489,7 +4558,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="194">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A194" s="8" t="s">
         <v>397</v>
       </c>
@@ -4500,7 +4569,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="195">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A195" s="8" t="s">
         <v>399</v>
       </c>
@@ -4511,7 +4580,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="196">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A196" s="8" t="s">
         <v>401</v>
       </c>
@@ -4522,7 +4591,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="197">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A197" s="8" t="s">
         <v>403</v>
       </c>
@@ -4533,7 +4602,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="198">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A198" s="8" t="s">
         <v>405</v>
       </c>
@@ -4544,7 +4613,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="199">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A199" s="8" t="s">
         <v>407</v>
       </c>
@@ -4555,7 +4624,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="200">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A200" s="8" t="s">
         <v>409</v>
       </c>
@@ -4566,7 +4635,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="201">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A201" s="8" t="s">
         <v>411</v>
       </c>
@@ -4577,7 +4646,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="202">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A202" s="8" t="s">
         <v>413</v>
       </c>
@@ -4588,7 +4657,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="203">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A203" s="8" t="s">
         <v>415</v>
       </c>
@@ -4599,7 +4668,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="204">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A204" s="8" t="s">
         <v>417</v>
       </c>
@@ -4610,7 +4679,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="205">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A205" s="8" t="s">
         <v>419</v>
       </c>
@@ -4621,7 +4690,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="206">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A206" s="8" t="s">
         <v>421</v>
       </c>
@@ -4632,7 +4701,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="207">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A207" s="8" t="s">
         <v>423</v>
       </c>
@@ -4643,7 +4712,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="208">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A208" s="8" t="s">
         <v>425</v>
       </c>
@@ -4654,7 +4723,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="209">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A209" s="8" t="s">
         <v>427</v>
       </c>
@@ -4665,7 +4734,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="210" ht="27">
+    <row r="210" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A210" s="9" t="s">
         <v>429</v>
       </c>
@@ -4676,7 +4745,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="211">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A211" s="8" t="s">
         <v>431</v>
       </c>
@@ -4687,7 +4756,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="212">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A212" s="8" t="s">
         <v>433</v>
       </c>
@@ -4698,7 +4767,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="213">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A213" s="8" t="s">
         <v>435</v>
       </c>
@@ -4709,7 +4778,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="214">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A214" s="8" t="s">
         <v>437</v>
       </c>
@@ -4720,7 +4789,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="215">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A215" s="8" t="s">
         <v>439</v>
       </c>
@@ -4731,7 +4800,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="216">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A216" s="8" t="s">
         <v>441</v>
       </c>
@@ -4742,7 +4811,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="217">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A217" s="8" t="s">
         <v>443</v>
       </c>
@@ -4753,7 +4822,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="218">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A218" s="8" t="s">
         <v>445</v>
       </c>
@@ -4764,7 +4833,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="219">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A219" s="8" t="s">
         <v>446</v>
       </c>
@@ -4775,7 +4844,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="220">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A220" s="8" t="s">
         <v>448</v>
       </c>
@@ -4786,7 +4855,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="221">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A221" s="8" t="s">
         <v>450</v>
       </c>
@@ -4797,7 +4866,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="222">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A222" s="8" t="s">
         <v>452</v>
       </c>
@@ -4808,7 +4877,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="223">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A223" s="8" t="s">
         <v>454</v>
       </c>
@@ -4819,7 +4888,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="224">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A224" s="8" t="s">
         <v>456</v>
       </c>
@@ -4830,7 +4899,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="225">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A225" s="8" t="s">
         <v>458</v>
       </c>
@@ -4841,7 +4910,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="226">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A226" s="8" t="s">
         <v>460</v>
       </c>
@@ -4852,7 +4921,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="227">
+    <row r="227" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A227" s="8" t="s">
         <v>462</v>
       </c>
@@ -4863,7 +4932,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="228">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A228" s="8" t="s">
         <v>464</v>
       </c>
@@ -4874,7 +4943,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="229">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A229" s="8" t="s">
         <v>466</v>
       </c>
@@ -4885,7 +4954,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="230">
+    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A230" s="8" t="s">
         <v>468</v>
       </c>
@@ -4896,7 +4965,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="231">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A231" s="8" t="s">
         <v>470</v>
       </c>
@@ -4907,7 +4976,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="232">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A232" s="8" t="s">
         <v>472</v>
       </c>
@@ -4918,7 +4987,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="233">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A233" s="8" t="s">
         <v>474</v>
       </c>
@@ -4929,7 +4998,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="234">
+    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A234" s="8" t="s">
         <v>476</v>
       </c>
@@ -4940,7 +5009,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="235">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A235" s="8" t="s">
         <v>478</v>
       </c>
@@ -4951,7 +5020,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="236">
+    <row r="236" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A236" s="8" t="s">
         <v>480</v>
       </c>
@@ -4962,7 +5031,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="237" ht="42">
+    <row r="237" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A237" s="9" t="s">
         <v>482</v>
       </c>
@@ -4973,7 +5042,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="238">
+    <row r="238" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A238" s="8" t="s">
         <v>484</v>
       </c>
@@ -4984,7 +5053,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="239">
+    <row r="239" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A239" s="8" t="s">
         <v>486</v>
       </c>
@@ -4995,7 +5064,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="240" ht="27">
+    <row r="240" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A240" s="9" t="s">
         <v>488</v>
       </c>
@@ -5006,7 +5075,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="241">
+    <row r="241" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A241" s="8" t="s">
         <v>490</v>
       </c>
@@ -5017,7 +5086,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="242">
+    <row r="242" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A242" s="8" t="s">
         <v>492</v>
       </c>
@@ -5028,7 +5097,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="243">
+    <row r="243" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A243" s="8" t="s">
         <v>494</v>
       </c>
@@ -5039,7 +5108,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="244">
+    <row r="244" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A244" s="8" t="s">
         <v>496</v>
       </c>
@@ -5050,7 +5119,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="245" ht="42">
+    <row r="245" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A245" s="9" t="s">
         <v>498</v>
       </c>
@@ -5061,7 +5130,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="246">
+    <row r="246" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A246" s="8" t="s">
         <v>500</v>
       </c>
@@ -5072,7 +5141,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="247" ht="42">
+    <row r="247" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A247" s="9" t="s">
         <v>502</v>
       </c>
@@ -5083,7 +5152,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="248">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A248" s="8" t="s">
         <v>504</v>
       </c>
@@ -5094,7 +5163,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="249">
+    <row r="249" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A249" s="8" t="s">
         <v>506</v>
       </c>
@@ -5105,7 +5174,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="250" ht="27">
+    <row r="250" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A250" s="9" t="s">
         <v>508</v>
       </c>
@@ -5116,7 +5185,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="251" ht="42">
+    <row r="251" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A251" s="9" t="s">
         <v>510</v>
       </c>
@@ -5127,7 +5196,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="252">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A252" s="8" t="s">
         <v>512</v>
       </c>
@@ -5138,7 +5207,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="253">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A253" s="8" t="s">
         <v>514</v>
       </c>
@@ -5149,7 +5218,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="254">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A254" s="8" t="s">
         <v>516</v>
       </c>
@@ -5160,7 +5229,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="255">
+    <row r="255" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A255" s="8" t="s">
         <v>518</v>
       </c>
@@ -5171,7 +5240,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="256" ht="27">
+    <row r="256" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A256" s="9" t="s">
         <v>520</v>
       </c>
@@ -5182,7 +5251,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="257">
+    <row r="257" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A257" s="8" t="s">
         <v>522</v>
       </c>
@@ -5193,7 +5262,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="258">
+    <row r="258" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A258" s="8" t="s">
         <v>524</v>
       </c>
@@ -5204,7 +5273,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="259">
+    <row r="259" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A259" s="8" t="s">
         <v>526</v>
       </c>
@@ -5215,7 +5284,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="260">
+    <row r="260" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A260" s="8" t="s">
         <v>528</v>
       </c>
@@ -5226,7 +5295,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="261">
+    <row r="261" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A261" s="8" t="s">
         <v>530</v>
       </c>
@@ -5237,7 +5306,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="262">
+    <row r="262" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A262" s="8" t="s">
         <v>532</v>
       </c>
@@ -5248,7 +5317,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="263">
+    <row r="263" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A263" s="8" t="s">
         <v>534</v>
       </c>
@@ -5259,7 +5328,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="264">
+    <row r="264" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A264" s="8" t="s">
         <v>536</v>
       </c>
@@ -5270,7 +5339,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="265">
+    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A265" s="8" t="s">
         <v>538</v>
       </c>
@@ -5281,7 +5350,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="266">
+    <row r="266" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A266" s="8" t="s">
         <v>540</v>
       </c>
@@ -5292,7 +5361,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="267">
+    <row r="267" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A267" s="8" t="s">
         <v>542</v>
       </c>
@@ -5303,7 +5372,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="268">
+    <row r="268" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A268" s="8" t="s">
         <v>544</v>
       </c>
@@ -5314,7 +5383,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="269">
+    <row r="269" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A269" s="8" t="s">
         <v>546</v>
       </c>
@@ -5325,7 +5394,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="270">
+    <row r="270" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A270" s="8" t="s">
         <v>548</v>
       </c>
@@ -5336,7 +5405,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="271">
+    <row r="271" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A271" s="8" t="s">
         <v>550</v>
       </c>
@@ -5347,7 +5416,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="272">
+    <row r="272" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A272" s="8" t="s">
         <v>552</v>
       </c>
@@ -5358,7 +5427,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="273">
+    <row r="273" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A273" s="8" t="s">
         <v>554</v>
       </c>
@@ -5369,7 +5438,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="274">
+    <row r="274" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A274" s="8" t="s">
         <v>556</v>
       </c>
@@ -5380,7 +5449,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="275">
+    <row r="275" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A275" s="8" t="s">
         <v>558</v>
       </c>
@@ -5391,7 +5460,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="276" ht="27">
+    <row r="276" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A276" s="9" t="s">
         <v>560</v>
       </c>
@@ -5402,7 +5471,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="277">
+    <row r="277" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A277" s="8" t="s">
         <v>562</v>
       </c>
@@ -5413,7 +5482,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="278">
+    <row r="278" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A278" s="8" t="s">
         <v>564</v>
       </c>
@@ -5424,7 +5493,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="279">
+    <row r="279" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A279" s="8" t="s">
         <v>566</v>
       </c>
@@ -5435,7 +5504,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="280" ht="27">
+    <row r="280" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A280" s="9" t="s">
         <v>568</v>
       </c>
@@ -5446,7 +5515,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="281">
+    <row r="281" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A281" s="8" t="s">
         <v>570</v>
       </c>
@@ -5457,7 +5526,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="282">
+    <row r="282" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A282" s="8" t="s">
         <v>572</v>
       </c>
@@ -5468,7 +5537,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="283">
+    <row r="283" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A283" s="9" t="s">
         <v>574</v>
       </c>
@@ -5479,7 +5548,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="284">
+    <row r="284" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A284" s="8" t="s">
         <v>576</v>
       </c>
@@ -5490,7 +5559,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="285" ht="27">
+    <row r="285" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A285" s="9" t="s">
         <v>578</v>
       </c>
@@ -5501,7 +5570,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="286">
+    <row r="286" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A286" s="3" t="s">
         <v>7</v>
       </c>
@@ -5512,7 +5581,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="287">
+    <row r="287" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A287" s="3" t="s">
         <v>4</v>
       </c>
@@ -5523,7 +5592,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="288">
+    <row r="288" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A288" s="3" t="s">
         <v>11</v>
       </c>
@@ -5534,7 +5603,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="289">
+    <row r="289" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A289" s="3" t="s">
         <v>6</v>
       </c>
@@ -5545,7 +5614,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="290">
+    <row r="290" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A290" s="3" t="s">
         <v>9</v>
       </c>
@@ -5556,7 +5625,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="291">
+    <row r="291" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A291" s="3" t="s">
         <v>5</v>
       </c>
@@ -5567,7 +5636,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="292">
+    <row r="292" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A292" s="3" t="s">
         <v>10</v>
       </c>
@@ -5578,7 +5647,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="293">
+    <row r="293" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A293" s="3" t="s">
         <v>8</v>
       </c>
@@ -5589,7 +5658,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="294">
+    <row r="294" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A294" s="3" t="s">
         <v>587</v>
       </c>
@@ -5600,7 +5669,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="295" ht="27">
+    <row r="295" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A295" s="2" t="s">
         <v>589</v>
       </c>
@@ -5611,7 +5680,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="296" ht="27">
+    <row r="296" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A296" s="2" t="s">
         <v>591</v>
       </c>
@@ -5622,7 +5691,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="297" ht="27">
+    <row r="297" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A297" s="2" t="s">
         <v>593</v>
       </c>
@@ -5633,7 +5702,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="298" ht="27">
+    <row r="298" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A298" s="2" t="s">
         <v>574</v>
       </c>
@@ -5644,7 +5713,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="299">
+    <row r="299" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A299" s="3" t="s">
         <v>576</v>
       </c>
@@ -5655,7 +5724,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="300" ht="27">
+    <row r="300" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A300" s="2" t="s">
         <v>578</v>
       </c>
@@ -5666,7 +5735,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="301">
+    <row r="301" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A301" s="3" t="s">
         <v>595</v>
       </c>
@@ -5677,7 +5746,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="302">
+    <row r="302" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A302" s="3" t="s">
         <v>596</v>
       </c>
@@ -5688,7 +5757,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="303">
+    <row r="303" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A303" s="3" t="s">
         <v>597</v>
       </c>
@@ -5699,7 +5768,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="304">
+    <row r="304" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A304" s="3" t="s">
         <v>598</v>
       </c>
@@ -5710,7 +5779,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="305">
+    <row r="305" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A305" s="3" t="s">
         <v>599</v>
       </c>
@@ -5721,7 +5790,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="306">
+    <row r="306" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A306" s="3" t="s">
         <v>600</v>
       </c>
@@ -5732,7 +5801,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="307">
+    <row r="307" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A307" s="3" t="s">
         <v>601</v>
       </c>
@@ -5743,7 +5812,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="308">
+    <row r="308" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A308" s="3" t="s">
         <v>602</v>
       </c>
@@ -5754,7 +5823,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="309">
+    <row r="309" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A309" s="3" t="s">
         <v>603</v>
       </c>
@@ -5765,7 +5834,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="310">
+    <row r="310" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A310" s="3" t="s">
         <v>604</v>
       </c>
@@ -5776,7 +5845,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="311">
+    <row r="311" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A311" s="3" t="s">
         <v>605</v>
       </c>
@@ -5787,7 +5856,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="312">
+    <row r="312" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A312" s="3" t="s">
         <v>607</v>
       </c>
@@ -5798,7 +5867,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="313">
+    <row r="313" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A313" s="3" t="s">
         <v>608</v>
       </c>
@@ -5809,7 +5878,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="314">
+    <row r="314" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A314" s="3" t="s">
         <v>609</v>
       </c>
@@ -5820,7 +5889,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="315">
+    <row r="315" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A315" s="3" t="s">
         <v>611</v>
       </c>
@@ -5831,7 +5900,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="316">
+    <row r="316" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A316" s="3" t="s">
         <v>613</v>
       </c>
@@ -5842,7 +5911,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="317">
+    <row r="317" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A317" s="3" t="s">
         <v>614</v>
       </c>
@@ -5853,7 +5922,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="318">
+    <row r="318" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A318" s="3" t="s">
         <v>615</v>
       </c>
@@ -5864,7 +5933,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="319">
+    <row r="319" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A319" s="3" t="s">
         <v>616</v>
       </c>
@@ -5875,7 +5944,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="320">
+    <row r="320" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A320" s="3" t="s">
         <v>617</v>
       </c>
@@ -5886,7 +5955,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="321">
+    <row r="321" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A321" s="3" t="s">
         <v>618</v>
       </c>
@@ -5897,7 +5966,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="322">
+    <row r="322" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A322" s="3" t="s">
         <v>619</v>
       </c>
@@ -5908,7 +5977,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="323">
+    <row r="323" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A323" s="3" t="s">
         <v>620</v>
       </c>
@@ -5919,7 +5988,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="324">
+    <row r="324" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A324" s="3" t="s">
         <v>621</v>
       </c>
@@ -5930,7 +5999,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="325">
+    <row r="325" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A325" s="3" t="s">
         <v>623</v>
       </c>
@@ -5941,7 +6010,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="326">
+    <row r="326" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A326" s="11" t="s">
         <v>620</v>
       </c>
@@ -5952,7 +6021,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="327">
+    <row r="327" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A327" s="11" t="s">
         <v>621</v>
       </c>
@@ -5963,7 +6032,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="328">
+    <row r="328" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A328" s="11" t="s">
         <v>623</v>
       </c>
@@ -5974,7 +6043,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="329">
+    <row r="329" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A329" s="10" t="s">
         <v>445</v>
       </c>
@@ -5985,19 +6054,192 @@
         <v>3</v>
       </c>
     </row>
-    <row r="330">
+    <row r="330" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A330" s="10" t="s">
+        <v>627</v>
+      </c>
+      <c r="B330" s="10" t="s">
         <v>628</v>
       </c>
-      <c r="B330" s="10" t="s">
-        <v>629</v>
-      </c>
       <c r="C330" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="331">
-      <c r="C331" s="6"/>
+    <row r="331" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A331" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B331" s="3" t="s">
+        <v>630</v>
+      </c>
+      <c r="C331" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="332" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A332" s="3" t="s">
+        <v>631</v>
+      </c>
+      <c r="B332" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="C332" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="333" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A333" s="3" t="s">
+        <v>633</v>
+      </c>
+      <c r="B333" s="3" t="s">
+        <v>634</v>
+      </c>
+      <c r="C333" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="334" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A334" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="B334" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="C334" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="335" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A335" s="3" t="s">
+        <v>637</v>
+      </c>
+      <c r="B335" s="3" t="s">
+        <v>638</v>
+      </c>
+      <c r="C335" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="336" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A336" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="B336" s="3" t="s">
+        <v>640</v>
+      </c>
+      <c r="C336" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="337" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A337" s="3" t="s">
+        <v>586</v>
+      </c>
+      <c r="B337" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="C337" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="338" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A338" s="3" t="s">
+        <v>583</v>
+      </c>
+      <c r="B338" s="3" t="s">
+        <v>642</v>
+      </c>
+      <c r="C338" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="339" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A339" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="B339" s="3" t="s">
+        <v>643</v>
+      </c>
+      <c r="C339" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="340" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A340" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B340" s="3" t="s">
+        <v>644</v>
+      </c>
+      <c r="C340" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="341" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A341" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="B341" s="3" t="s">
+        <v>645</v>
+      </c>
+      <c r="C341" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="342" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A342" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="B342" s="3" t="s">
+        <v>646</v>
+      </c>
+      <c r="C342" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="343" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A343" s="3" t="s">
+        <v>582</v>
+      </c>
+      <c r="B343" s="3" t="s">
+        <v>647</v>
+      </c>
+      <c r="C343" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="344" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A344" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="B344" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="C344" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="345" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A345" s="3" t="s">
+        <v>650</v>
+      </c>
+      <c r="B345" s="3" t="s">
+        <v>651</v>
+      </c>
+      <c r="C345" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="346" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A346" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="B346" s="3" t="s">
+        <v>653</v>
+      </c>
+      <c r="C346" s="6" t="s">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6647,6 +6889,38 @@
     <hyperlink ref="B327" r:id="rId644" tooltip="https://www.addact.net/portfolio" display="https://www.addact.net/portfolio" xr:uid="{5B40D3C6-D44A-4551-86D7-F50A5C3526A1}"/>
     <hyperlink ref="A328" r:id="rId645" tooltip="https://www.addact.net/addact-next-chapter-reveal" display="https://www.addact.net/addact-next-chapter-reveal" xr:uid="{93DAE1B6-838E-4B70-B21B-9BAAECE8FFC8}"/>
     <hyperlink ref="B328" r:id="rId646" tooltip="https://www.addact.net/addact-next-chapter-reveal" display="https://www.addact.net/addact-next-chapter-reveal" xr:uid="{6A8CD1F8-1B5E-493A-B705-EEB97D336605}"/>
+    <hyperlink ref="A331" r:id="rId647" display="https://www.addact.net/sitecore-cms-development" xr:uid="{79F58A88-0562-4B8A-A19D-A0B31FD36CCA}"/>
+    <hyperlink ref="A332" r:id="rId648" display="https://www.addact.net/umbraco-cms-development" xr:uid="{6F2FB189-5CA1-494F-98FE-BF3CC5D62B9A}"/>
+    <hyperlink ref="A333" r:id="rId649" display="https://www.addact.net/strapi-cms-development" xr:uid="{8C044089-9761-4A1C-92E9-23EB7ACB11AE}"/>
+    <hyperlink ref="A334" r:id="rId650" display="https://www.addact.net/kentico-cms-development" xr:uid="{806716F4-7567-4D5D-9670-00B30EF37D57}"/>
+    <hyperlink ref="A335" r:id="rId651" display="https://www.addact.net/contentful-cms-development" xr:uid="{1F0958B9-26E3-4777-965D-F3CD1E48E4A0}"/>
+    <hyperlink ref="A336" r:id="rId652" display="https://www.addact.net/contentstack-cms-development" xr:uid="{D0DA70CC-6A63-4720-883E-2E5A41C7E604}"/>
+    <hyperlink ref="A337" r:id="rId653" display="https://www.addact.net/sitecore-cms-development/sitecore-support-and-maintenance-services" xr:uid="{0BC580AD-E16E-4E10-B2B7-A73838A9263B}"/>
+    <hyperlink ref="A338" r:id="rId654" display="https://www.addact.net/sitecore-cms-development/sitecore-consulting-services" xr:uid="{F81C4BDC-E0F9-4C6C-8944-05F1A7DCA719}"/>
+    <hyperlink ref="A339" r:id="rId655" display="https://www.addact.net/sitecore-cms-development/sitecore-xm-cloud-services" xr:uid="{FCF7990F-A26C-413A-AD3A-DA5BA78BF082}"/>
+    <hyperlink ref="A340" r:id="rId656" display="https://www.addact.net/sitecore-cms-development/sitecore-platform-integrations" xr:uid="{65D37170-ED72-43CF-AEBD-7F3435FB85E6}"/>
+    <hyperlink ref="A341" r:id="rId657" display="https://www.addact.net/sitecore-cms-development/sitecore-audit-service" xr:uid="{7A62116B-CFB2-44F6-940E-DF6FAF2AC57C}"/>
+    <hyperlink ref="A342" r:id="rId658" display="https://www.addact.net/sitecore-cms-development/sitecore-platform-upgrade-services" xr:uid="{6E7449B6-C873-496F-BC46-ECB2CEEAD5B9}"/>
+    <hyperlink ref="B331" r:id="rId659" display="https://www.addact.net/development-design/cms-development/sitecore" xr:uid="{03CAC35C-C6DF-48B0-98ED-E1ECFD02D7DB}"/>
+    <hyperlink ref="B332" r:id="rId660" display="https://www.addact.net/development-design/cms-development/umbraco" xr:uid="{B2AC881C-CF16-4C0D-9B22-67B82C3B7847}"/>
+    <hyperlink ref="B333" r:id="rId661" display="https://www.addact.net/development-design/cms-development/strapi" xr:uid="{6FF2A706-9818-414D-BF0D-3CDA19D81652}"/>
+    <hyperlink ref="B334" r:id="rId662" display="https://www.addact.net/development-design/cms-development/kentico" xr:uid="{6A755B5A-829F-4200-8475-983FF9616472}"/>
+    <hyperlink ref="B335" r:id="rId663" display="https://www.addact.net/development-design/cms-development/contentful" xr:uid="{9E54DCE4-7D0E-4A28-B7AD-333BE6E5B486}"/>
+    <hyperlink ref="B336" r:id="rId664" display="https://www.addact.net/development-design/cms-development/contentstack" xr:uid="{E7B11DEB-ABD7-435A-8E99-9DA7FAFE2682}"/>
+    <hyperlink ref="B337" r:id="rId665" display="https://www.addact.net/development-design/cms-development/sitecore/support-and-maintenance" xr:uid="{66E59B3A-6832-4C7C-8E02-0FAB0C06C6F1}"/>
+    <hyperlink ref="B338" r:id="rId666" display="https://www.addact.net/development-design/cms-development/sitecore/consulting-services" xr:uid="{51AC340A-A7A9-426D-97A1-404703E5A519}"/>
+    <hyperlink ref="B339" r:id="rId667" display="https://www.addact.net/development-design/cms-development/sitecore/sitecore-ai" xr:uid="{83828BC0-2BBF-45A5-BBB2-8E3BAFD52F13}"/>
+    <hyperlink ref="B340" r:id="rId668" display="https://www.addact.net/development-design/cms-development/sitecore/platform-integrations" xr:uid="{06BB026C-8ECE-4815-A8F3-6E2C7BCB3C8E}"/>
+    <hyperlink ref="B341" r:id="rId669" display="https://www.addact.net/development-design/cms-development/sitecore/audit-service" xr:uid="{82634523-5B98-4CE0-8A3E-DBA3E1A63834}"/>
+    <hyperlink ref="B342" r:id="rId670" display="https://www.addact.net/development-design/cms-development/sitecore/platform-upgrade" xr:uid="{D49F6B1D-D3A0-4794-B5E0-9AE7234B0AAA}"/>
+    <hyperlink ref="A343" r:id="rId671" display="https://www.addact.net/sitecore-cms-development/hire-sitecore-developer" xr:uid="{303C74B5-0221-48C1-9C36-AEAD1964A885}"/>
+    <hyperlink ref="A344" r:id="rId672" display="https://www.addact.net/umbraco-cms-development/hire-umbraco-developer" xr:uid="{18038A8B-7031-4027-BF59-4501C8A31600}"/>
+    <hyperlink ref="A345" r:id="rId673" display="https://www.addact.net/strapi-cms-development/hire-strapi-developer" xr:uid="{5BCF3315-481F-4436-AD1D-B0B8C8227D3D}"/>
+    <hyperlink ref="A346" r:id="rId674" display="https://www.addact.net/kentico-cms-development/hire-kentico-developer" xr:uid="{2E157BB3-0B5F-4E7F-B622-EB18AC4C7A03}"/>
+    <hyperlink ref="B343" r:id="rId675" display="https://www.addact.net/hire-experts/sitecore-developer" xr:uid="{94CDABEA-997A-44FE-B798-DE3303A294EA}"/>
+    <hyperlink ref="B344" r:id="rId676" display="https://www.addact.net/hire-expert/umbraco-developer" xr:uid="{FCDDBDCE-1843-4317-94E4-1B70EB9DBF04}"/>
+    <hyperlink ref="B345" r:id="rId677" display="https://www.addact.net/hire-expert/strapi-developer" xr:uid="{E4D49E07-6A2F-4A09-AC25-A47B8CB158B6}"/>
+    <hyperlink ref="B346" r:id="rId678" display="https://www.addact.net/hire-experts/kentico-developer" xr:uid="{0DE63966-9454-4E7F-9874-4FB7691962D7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: remove unuse packages and remove unuse route component
</commit_message>
<xml_diff>
--- a/addact/public/redirects.xlsx
+++ b/addact/public/redirects.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\Addact-Revamp\addact\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Addact-Revamp\addact\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D088DA5C-078C-4D7F-A278-20525E1ED177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E5271F-47B8-4814-8971-45A67DBCDB97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5F6600C6-C08A-47D2-B3C8-F7A43562057B}"/>
+    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{5F6600C6-C08A-47D2-B3C8-F7A43562057B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="654">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="655">
   <si>
     <t>source</t>
   </si>
@@ -1998,6 +1998,9 @@
   </si>
   <si>
     <t>/hire-experts/kentico-developer</t>
+  </si>
+  <si>
+    <t>/hire-certified-sitecore-developer</t>
   </si>
 </sst>
 </file>
@@ -2427,7 +2430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C59FA00F-2D8F-4BC7-B234-D60C0BA408AE}">
-  <dimension ref="A1:C346"/>
+  <dimension ref="A1:C347"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="107.44140625" customWidth="1"/>
@@ -6238,6 +6241,17 @@
         <v>653</v>
       </c>
       <c r="C346" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="347" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A347" t="s">
+        <v>654</v>
+      </c>
+      <c r="B347" t="s">
+        <v>630</v>
+      </c>
+      <c r="C347" s="6" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Squashed commit of the following:
commit ac93a2b162f19f5fb67acc9aa540324596b1a467
Merge: 969bd0e 50cfd26
Author: devam chaudhari <devam@addact.net>
Date:   Thu Mar 26 18:10:15 2026 +0530

    Merge pull request #648 from Addact-Devops/fix/bug-20-03

    Fix/bug 20 03

commit 50cfd267bcb88a5a6d6594ddfad6b2a805cb9a58
Author: devam <devam@addact.net>
Date:   Thu Mar 26 18:08:26 2026 +0530

    fix: added fix code format and save all file for the format

commit 4ac979e31da593a8c6a80290f4832b66bd9c5952
Author: devam <devam@addact.net>
Date:   Thu Mar 26 17:06:57 2026 +0530

    fix: remove unuse packages and remove unuse route component
</commit_message>
<xml_diff>
--- a/addact/public/redirects.xlsx
+++ b/addact/public/redirects.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\Addact-Revamp\addact\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Addact-Revamp\addact\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D088DA5C-078C-4D7F-A278-20525E1ED177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E5271F-47B8-4814-8971-45A67DBCDB97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5F6600C6-C08A-47D2-B3C8-F7A43562057B}"/>
+    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{5F6600C6-C08A-47D2-B3C8-F7A43562057B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="654">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="655">
   <si>
     <t>source</t>
   </si>
@@ -1998,6 +1998,9 @@
   </si>
   <si>
     <t>/hire-experts/kentico-developer</t>
+  </si>
+  <si>
+    <t>/hire-certified-sitecore-developer</t>
   </si>
 </sst>
 </file>
@@ -2427,7 +2430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C59FA00F-2D8F-4BC7-B234-D60C0BA408AE}">
-  <dimension ref="A1:C346"/>
+  <dimension ref="A1:C347"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="107.44140625" customWidth="1"/>
@@ -6238,6 +6241,17 @@
         <v>653</v>
       </c>
       <c r="C346" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="347" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A347" t="s">
+        <v>654</v>
+      </c>
+      <c r="B347" t="s">
+        <v>630</v>
+      </c>
+      <c r="C347" s="6" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: added new redirect links
</commit_message>
<xml_diff>
--- a/addact/public/redirects.xlsx
+++ b/addact/public/redirects.xlsx
@@ -8,35 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Addact-Revamp\addact\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E5271F-47B8-4814-8971-45A67DBCDB97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6EE1969-9EDA-46C7-BBCD-4FBAF73A9D5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{5F6600C6-C08A-47D2-B3C8-F7A43562057B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="659">
   <si>
     <t>source</t>
   </si>
@@ -2001,13 +1990,25 @@
   </si>
   <si>
     <t>/hire-certified-sitecore-developer</t>
+  </si>
+  <si>
+    <t>/contact</t>
+  </si>
+  <si>
+    <t>/contact-us</t>
+  </si>
+  <si>
+    <t>/project-cost-estimator</t>
+  </si>
+  <si>
+    <t>/project-cost-estimators</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2038,6 +2039,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -2066,7 +2074,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2095,6 +2103,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2430,15 +2439,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C59FA00F-2D8F-4BC7-B234-D60C0BA408AE}">
-  <dimension ref="A1:C347"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C349"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="107.44140625" customWidth="1"/>
-    <col min="2" max="2" width="83.109375" customWidth="1"/>
-    <col min="3" max="3" width="14.21875" style="7" customWidth="1"/>
+    <col min="1" max="1" width="107.42578125" customWidth="1"/>
+    <col min="2" max="2" width="83.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2449,7 +2458,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
@@ -2460,7 +2469,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>16</v>
       </c>
@@ -2471,7 +2480,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>18</v>
       </c>
@@ -2482,7 +2491,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>20</v>
       </c>
@@ -2493,7 +2502,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>22</v>
       </c>
@@ -2504,7 +2513,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>24</v>
       </c>
@@ -2515,7 +2524,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>26</v>
       </c>
@@ -2526,7 +2535,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>28</v>
       </c>
@@ -2537,7 +2546,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>30</v>
       </c>
@@ -2548,7 +2557,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>32</v>
       </c>
@@ -2559,7 +2568,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>34</v>
       </c>
@@ -2570,7 +2579,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>35</v>
       </c>
@@ -2581,7 +2590,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>37</v>
       </c>
@@ -2592,7 +2601,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>39</v>
       </c>
@@ -2603,7 +2612,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>41</v>
       </c>
@@ -2614,7 +2623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>43</v>
       </c>
@@ -2625,7 +2634,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>45</v>
       </c>
@@ -2636,7 +2645,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>47</v>
       </c>
@@ -2647,7 +2656,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
         <v>49</v>
       </c>
@@ -2658,7 +2667,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
         <v>51</v>
       </c>
@@ -2669,7 +2678,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
         <v>53</v>
       </c>
@@ -2680,7 +2689,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
         <v>55</v>
       </c>
@@ -2691,7 +2700,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>57</v>
       </c>
@@ -2702,7 +2711,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>59</v>
       </c>
@@ -2713,7 +2722,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>61</v>
       </c>
@@ -2724,7 +2733,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
         <v>63</v>
       </c>
@@ -2735,7 +2744,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>65</v>
       </c>
@@ -2746,7 +2755,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
         <v>67</v>
       </c>
@@ -2757,7 +2766,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>69</v>
       </c>
@@ -2768,7 +2777,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
         <v>71</v>
       </c>
@@ -2779,7 +2788,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>73</v>
       </c>
@@ -2790,7 +2799,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
         <v>75</v>
       </c>
@@ -2801,7 +2810,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
         <v>77</v>
       </c>
@@ -2812,7 +2821,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
         <v>79</v>
       </c>
@@ -2823,7 +2832,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
         <v>81</v>
       </c>
@@ -2834,7 +2843,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
         <v>83</v>
       </c>
@@ -2845,7 +2854,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
         <v>85</v>
       </c>
@@ -2856,7 +2865,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
         <v>87</v>
       </c>
@@ -2867,7 +2876,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
         <v>89</v>
       </c>
@@ -2878,7 +2887,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
         <v>91</v>
       </c>
@@ -2889,7 +2898,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
         <v>93</v>
       </c>
@@ -2900,7 +2909,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="9" t="s">
         <v>95</v>
       </c>
@@ -2911,7 +2920,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
         <v>97</v>
       </c>
@@ -2922,7 +2931,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
         <v>99</v>
       </c>
@@ -2933,7 +2942,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="8" t="s">
         <v>101</v>
       </c>
@@ -2944,7 +2953,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
         <v>103</v>
       </c>
@@ -2955,7 +2964,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
         <v>105</v>
       </c>
@@ -2966,7 +2975,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
         <v>107</v>
       </c>
@@ -2977,7 +2986,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
         <v>109</v>
       </c>
@@ -2988,7 +2997,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
         <v>111</v>
       </c>
@@ -2999,7 +3008,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
         <v>113</v>
       </c>
@@ -3010,7 +3019,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
         <v>115</v>
       </c>
@@ -3021,7 +3030,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="8" t="s">
         <v>117</v>
       </c>
@@ -3032,7 +3041,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
         <v>119</v>
       </c>
@@ -3043,7 +3052,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
         <v>121</v>
       </c>
@@ -3054,7 +3063,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
         <v>123</v>
       </c>
@@ -3065,7 +3074,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
         <v>125</v>
       </c>
@@ -3076,7 +3085,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
         <v>127</v>
       </c>
@@ -3087,7 +3096,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="8" t="s">
         <v>129</v>
       </c>
@@ -3098,7 +3107,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
         <v>131</v>
       </c>
@@ -3109,7 +3118,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="8" t="s">
         <v>133</v>
       </c>
@@ -3120,7 +3129,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
         <v>135</v>
       </c>
@@ -3131,7 +3140,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="9" t="s">
         <v>137</v>
       </c>
@@ -3142,7 +3151,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
         <v>139</v>
       </c>
@@ -3153,7 +3162,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="8" t="s">
         <v>141</v>
       </c>
@@ -3164,7 +3173,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
         <v>143</v>
       </c>
@@ -3175,7 +3184,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="8" t="s">
         <v>145</v>
       </c>
@@ -3186,7 +3195,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
         <v>147</v>
       </c>
@@ -3197,7 +3206,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="8" t="s">
         <v>149</v>
       </c>
@@ -3208,7 +3217,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="9" t="s">
         <v>151</v>
       </c>
@@ -3219,7 +3228,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="9" t="s">
         <v>153</v>
       </c>
@@ -3230,7 +3239,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
         <v>155</v>
       </c>
@@ -3241,7 +3250,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="8" t="s">
         <v>157</v>
       </c>
@@ -3252,7 +3261,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="9" t="s">
         <v>159</v>
       </c>
@@ -3263,7 +3272,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="8" t="s">
         <v>161</v>
       </c>
@@ -3274,7 +3283,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
         <v>163</v>
       </c>
@@ -3285,7 +3294,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="8" t="s">
         <v>165</v>
       </c>
@@ -3296,7 +3305,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
         <v>167</v>
       </c>
@@ -3307,7 +3316,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="8" t="s">
         <v>169</v>
       </c>
@@ -3318,7 +3327,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
         <v>171</v>
       </c>
@@ -3329,7 +3338,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="8" t="s">
         <v>173</v>
       </c>
@@ -3340,7 +3349,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
         <v>175</v>
       </c>
@@ -3351,7 +3360,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="8" t="s">
         <v>177</v>
       </c>
@@ -3362,7 +3371,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
         <v>179</v>
       </c>
@@ -3373,7 +3382,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="8" t="s">
         <v>181</v>
       </c>
@@ -3384,7 +3393,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
         <v>183</v>
       </c>
@@ -3395,7 +3404,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="8" t="s">
         <v>185</v>
       </c>
@@ -3406,7 +3415,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
         <v>187</v>
       </c>
@@ -3417,7 +3426,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="8" t="s">
         <v>189</v>
       </c>
@@ -3428,7 +3437,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
         <v>191</v>
       </c>
@@ -3439,7 +3448,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="8" t="s">
         <v>193</v>
       </c>
@@ -3450,7 +3459,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
         <v>195</v>
       </c>
@@ -3461,7 +3470,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="8" t="s">
         <v>197</v>
       </c>
@@ -3472,7 +3481,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="9" t="s">
         <v>199</v>
       </c>
@@ -3483,7 +3492,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="8" t="s">
         <v>201</v>
       </c>
@@ -3494,7 +3503,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
         <v>203</v>
       </c>
@@ -3505,7 +3514,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" s="8" t="s">
         <v>205</v>
       </c>
@@ -3516,7 +3525,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" s="9" t="s">
         <v>207</v>
       </c>
@@ -3527,7 +3536,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" s="8" t="s">
         <v>209</v>
       </c>
@@ -3538,7 +3547,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
         <v>211</v>
       </c>
@@ -3549,7 +3558,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" s="8" t="s">
         <v>213</v>
       </c>
@@ -3560,7 +3569,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
         <v>215</v>
       </c>
@@ -3571,7 +3580,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" s="8" t="s">
         <v>217</v>
       </c>
@@ -3582,7 +3591,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" s="8" t="s">
         <v>219</v>
       </c>
@@ -3593,7 +3602,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" s="8" t="s">
         <v>221</v>
       </c>
@@ -3604,7 +3613,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" s="8" t="s">
         <v>223</v>
       </c>
@@ -3615,7 +3624,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" s="8" t="s">
         <v>225</v>
       </c>
@@ -3626,7 +3635,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" s="8" t="s">
         <v>227</v>
       </c>
@@ -3637,7 +3646,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" s="8" t="s">
         <v>229</v>
       </c>
@@ -3648,7 +3657,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" s="8" t="s">
         <v>231</v>
       </c>
@@ -3659,7 +3668,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" s="8" t="s">
         <v>233</v>
       </c>
@@ -3670,7 +3679,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
         <v>235</v>
       </c>
@@ -3681,7 +3690,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" s="8" t="s">
         <v>237</v>
       </c>
@@ -3692,7 +3701,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" s="8" t="s">
         <v>239</v>
       </c>
@@ -3703,7 +3712,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" s="8" t="s">
         <v>241</v>
       </c>
@@ -3714,7 +3723,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" s="9" t="s">
         <v>243</v>
       </c>
@@ -3725,7 +3734,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" s="8" t="s">
         <v>245</v>
       </c>
@@ -3736,7 +3745,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" s="8" t="s">
         <v>247</v>
       </c>
@@ -3747,7 +3756,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" s="8" t="s">
         <v>249</v>
       </c>
@@ -3758,7 +3767,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
         <v>251</v>
       </c>
@@ -3769,7 +3778,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" s="9" t="s">
         <v>253</v>
       </c>
@@ -3780,7 +3789,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" s="8" t="s">
         <v>255</v>
       </c>
@@ -3791,7 +3800,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" s="8" t="s">
         <v>257</v>
       </c>
@@ -3802,7 +3811,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" s="8" t="s">
         <v>259</v>
       </c>
@@ -3813,7 +3822,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" s="8" t="s">
         <v>261</v>
       </c>
@@ -3824,7 +3833,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" s="8" t="s">
         <v>263</v>
       </c>
@@ -3835,7 +3844,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" s="8" t="s">
         <v>265</v>
       </c>
@@ -3846,7 +3855,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" s="8" t="s">
         <v>267</v>
       </c>
@@ -3857,7 +3866,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" s="8" t="s">
         <v>269</v>
       </c>
@@ -3868,7 +3877,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" s="8" t="s">
         <v>271</v>
       </c>
@@ -3879,7 +3888,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" s="8" t="s">
         <v>273</v>
       </c>
@@ -3890,7 +3899,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" s="8" t="s">
         <v>275</v>
       </c>
@@ -3901,7 +3910,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" s="8" t="s">
         <v>277</v>
       </c>
@@ -3912,7 +3921,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" s="8" t="s">
         <v>279</v>
       </c>
@@ -3923,7 +3932,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" s="8" t="s">
         <v>281</v>
       </c>
@@ -3934,7 +3943,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" s="8" t="s">
         <v>283</v>
       </c>
@@ -3945,7 +3954,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" s="8" t="s">
         <v>285</v>
       </c>
@@ -3956,7 +3965,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A139" s="9" t="s">
         <v>287</v>
       </c>
@@ -3967,7 +3976,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" s="8" t="s">
         <v>289</v>
       </c>
@@ -3978,7 +3987,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" s="8" t="s">
         <v>291</v>
       </c>
@@ -3989,7 +3998,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" s="8" t="s">
         <v>293</v>
       </c>
@@ -4000,7 +4009,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" s="8" t="s">
         <v>295</v>
       </c>
@@ -4011,7 +4020,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" s="8" t="s">
         <v>297</v>
       </c>
@@ -4022,7 +4031,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" s="8" t="s">
         <v>299</v>
       </c>
@@ -4033,7 +4042,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" s="8" t="s">
         <v>301</v>
       </c>
@@ -4044,7 +4053,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" s="8" t="s">
         <v>303</v>
       </c>
@@ -4055,7 +4064,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" s="8" t="s">
         <v>305</v>
       </c>
@@ -4066,7 +4075,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" s="8" t="s">
         <v>307</v>
       </c>
@@ -4077,7 +4086,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" s="8" t="s">
         <v>309</v>
       </c>
@@ -4088,7 +4097,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" s="8" t="s">
         <v>311</v>
       </c>
@@ -4099,7 +4108,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" s="8" t="s">
         <v>313</v>
       </c>
@@ -4110,7 +4119,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" s="8" t="s">
         <v>315</v>
       </c>
@@ -4121,7 +4130,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" s="8" t="s">
         <v>317</v>
       </c>
@@ -4132,7 +4141,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" s="8" t="s">
         <v>319</v>
       </c>
@@ -4143,7 +4152,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" s="8" t="s">
         <v>321</v>
       </c>
@@ -4154,7 +4163,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" s="8" t="s">
         <v>323</v>
       </c>
@@ -4165,7 +4174,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" s="8" t="s">
         <v>325</v>
       </c>
@@ -4176,7 +4185,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" s="8" t="s">
         <v>327</v>
       </c>
@@ -4187,7 +4196,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" s="8" t="s">
         <v>329</v>
       </c>
@@ -4198,7 +4207,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" s="8" t="s">
         <v>331</v>
       </c>
@@ -4209,7 +4218,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" s="8" t="s">
         <v>333</v>
       </c>
@@ -4220,7 +4229,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" s="8" t="s">
         <v>335</v>
       </c>
@@ -4231,7 +4240,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" s="8" t="s">
         <v>337</v>
       </c>
@@ -4242,7 +4251,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" s="8" t="s">
         <v>339</v>
       </c>
@@ -4253,7 +4262,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" s="8" t="s">
         <v>341</v>
       </c>
@@ -4264,7 +4273,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" s="8" t="s">
         <v>343</v>
       </c>
@@ -4275,7 +4284,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" s="8" t="s">
         <v>345</v>
       </c>
@@ -4286,7 +4295,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" s="8" t="s">
         <v>347</v>
       </c>
@@ -4297,7 +4306,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" s="8" t="s">
         <v>349</v>
       </c>
@@ -4308,7 +4317,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" s="8" t="s">
         <v>351</v>
       </c>
@@ -4319,7 +4328,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" s="8" t="s">
         <v>353</v>
       </c>
@@ -4330,7 +4339,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" s="8" t="s">
         <v>355</v>
       </c>
@@ -4341,7 +4350,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" s="8" t="s">
         <v>357</v>
       </c>
@@ -4352,7 +4361,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" s="8" t="s">
         <v>359</v>
       </c>
@@ -4363,7 +4372,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" s="8" t="s">
         <v>361</v>
       </c>
@@ -4374,7 +4383,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="8" t="s">
         <v>363</v>
       </c>
@@ -4385,7 +4394,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="8" t="s">
         <v>365</v>
       </c>
@@ -4396,7 +4405,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="8" t="s">
         <v>367</v>
       </c>
@@ -4407,7 +4416,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="8" t="s">
         <v>369</v>
       </c>
@@ -4418,7 +4427,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="8" t="s">
         <v>371</v>
       </c>
@@ -4429,7 +4438,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="8" t="s">
         <v>373</v>
       </c>
@@ -4440,7 +4449,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="183" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A183" s="9" t="s">
         <v>375</v>
       </c>
@@ -4451,7 +4460,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="8" t="s">
         <v>377</v>
       </c>
@@ -4462,7 +4471,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="8" t="s">
         <v>379</v>
       </c>
@@ -4473,7 +4482,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="8" t="s">
         <v>381</v>
       </c>
@@ -4484,7 +4493,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="8" t="s">
         <v>383</v>
       </c>
@@ -4495,7 +4504,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="8" t="s">
         <v>385</v>
       </c>
@@ -4506,7 +4515,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="8" t="s">
         <v>387</v>
       </c>
@@ -4517,7 +4526,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="8" t="s">
         <v>389</v>
       </c>
@@ -4528,7 +4537,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="8" t="s">
         <v>391</v>
       </c>
@@ -4539,7 +4548,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="8" t="s">
         <v>393</v>
       </c>
@@ -4550,7 +4559,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" s="8" t="s">
         <v>395</v>
       </c>
@@ -4561,7 +4570,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" s="8" t="s">
         <v>397</v>
       </c>
@@ -4572,7 +4581,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" s="8" t="s">
         <v>399</v>
       </c>
@@ -4583,7 +4592,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" s="8" t="s">
         <v>401</v>
       </c>
@@ -4594,7 +4603,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" s="8" t="s">
         <v>403</v>
       </c>
@@ -4605,7 +4614,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" s="8" t="s">
         <v>405</v>
       </c>
@@ -4616,7 +4625,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" s="8" t="s">
         <v>407</v>
       </c>
@@ -4627,7 +4636,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" s="8" t="s">
         <v>409</v>
       </c>
@@ -4638,7 +4647,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="8" t="s">
         <v>411</v>
       </c>
@@ -4649,7 +4658,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" s="8" t="s">
         <v>413</v>
       </c>
@@ -4660,7 +4669,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" s="8" t="s">
         <v>415</v>
       </c>
@@ -4671,7 +4680,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" s="8" t="s">
         <v>417</v>
       </c>
@@ -4682,7 +4691,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" s="8" t="s">
         <v>419</v>
       </c>
@@ -4693,7 +4702,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" s="8" t="s">
         <v>421</v>
       </c>
@@ -4704,7 +4713,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" s="8" t="s">
         <v>423</v>
       </c>
@@ -4715,7 +4724,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" s="8" t="s">
         <v>425</v>
       </c>
@@ -4726,7 +4735,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" s="8" t="s">
         <v>427</v>
       </c>
@@ -4737,7 +4746,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="210" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A210" s="9" t="s">
         <v>429</v>
       </c>
@@ -4748,7 +4757,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" s="8" t="s">
         <v>431</v>
       </c>
@@ -4759,7 +4768,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" s="8" t="s">
         <v>433</v>
       </c>
@@ -4770,7 +4779,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" s="8" t="s">
         <v>435</v>
       </c>
@@ -4781,7 +4790,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" s="8" t="s">
         <v>437</v>
       </c>
@@ -4792,7 +4801,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" s="8" t="s">
         <v>439</v>
       </c>
@@ -4803,7 +4812,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" s="8" t="s">
         <v>441</v>
       </c>
@@ -4814,7 +4823,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" s="8" t="s">
         <v>443</v>
       </c>
@@ -4825,7 +4834,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" s="8" t="s">
         <v>445</v>
       </c>
@@ -4836,7 +4845,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" s="8" t="s">
         <v>446</v>
       </c>
@@ -4847,7 +4856,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" s="8" t="s">
         <v>448</v>
       </c>
@@ -4858,7 +4867,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" s="8" t="s">
         <v>450</v>
       </c>
@@ -4869,7 +4878,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" s="8" t="s">
         <v>452</v>
       </c>
@@ -4880,7 +4889,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" s="8" t="s">
         <v>454</v>
       </c>
@@ -4891,7 +4900,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" s="8" t="s">
         <v>456</v>
       </c>
@@ -4902,7 +4911,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" s="8" t="s">
         <v>458</v>
       </c>
@@ -4913,7 +4922,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" s="8" t="s">
         <v>460</v>
       </c>
@@ -4924,7 +4933,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227" s="8" t="s">
         <v>462</v>
       </c>
@@ -4935,7 +4944,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" s="8" t="s">
         <v>464</v>
       </c>
@@ -4946,7 +4955,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" s="8" t="s">
         <v>466</v>
       </c>
@@ -4957,7 +4966,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" s="8" t="s">
         <v>468</v>
       </c>
@@ -4968,7 +4977,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" s="8" t="s">
         <v>470</v>
       </c>
@@ -4979,7 +4988,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232" s="8" t="s">
         <v>472</v>
       </c>
@@ -4990,7 +4999,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" s="8" t="s">
         <v>474</v>
       </c>
@@ -5001,7 +5010,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" s="8" t="s">
         <v>476</v>
       </c>
@@ -5012,7 +5021,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235" s="8" t="s">
         <v>478</v>
       </c>
@@ -5023,7 +5032,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" s="8" t="s">
         <v>480</v>
       </c>
@@ -5034,7 +5043,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="237" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A237" s="9" t="s">
         <v>482</v>
       </c>
@@ -5045,7 +5054,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" s="8" t="s">
         <v>484</v>
       </c>
@@ -5056,7 +5065,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" s="8" t="s">
         <v>486</v>
       </c>
@@ -5067,7 +5076,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A240" s="9" t="s">
         <v>488</v>
       </c>
@@ -5078,7 +5087,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="241" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" s="8" t="s">
         <v>490</v>
       </c>
@@ -5089,7 +5098,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="242" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" s="8" t="s">
         <v>492</v>
       </c>
@@ -5100,7 +5109,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="243" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" s="8" t="s">
         <v>494</v>
       </c>
@@ -5111,7 +5120,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" s="8" t="s">
         <v>496</v>
       </c>
@@ -5122,7 +5131,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="245" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A245" s="9" t="s">
         <v>498</v>
       </c>
@@ -5133,7 +5142,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246" s="8" t="s">
         <v>500</v>
       </c>
@@ -5144,7 +5153,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="247" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A247" s="9" t="s">
         <v>502</v>
       </c>
@@ -5155,7 +5164,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="248" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" s="8" t="s">
         <v>504</v>
       </c>
@@ -5166,7 +5175,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249" s="8" t="s">
         <v>506</v>
       </c>
@@ -5177,7 +5186,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="250" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A250" s="9" t="s">
         <v>508</v>
       </c>
@@ -5188,7 +5197,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="251" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A251" s="9" t="s">
         <v>510</v>
       </c>
@@ -5199,7 +5208,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="252" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" s="8" t="s">
         <v>512</v>
       </c>
@@ -5210,7 +5219,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="253" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" s="8" t="s">
         <v>514</v>
       </c>
@@ -5221,7 +5230,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="254" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" s="8" t="s">
         <v>516</v>
       </c>
@@ -5232,7 +5241,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="255" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" s="8" t="s">
         <v>518</v>
       </c>
@@ -5243,7 +5252,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="256" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A256" s="9" t="s">
         <v>520</v>
       </c>
@@ -5254,7 +5263,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" s="8" t="s">
         <v>522</v>
       </c>
@@ -5265,7 +5274,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="258" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" s="8" t="s">
         <v>524</v>
       </c>
@@ -5276,7 +5285,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259" s="8" t="s">
         <v>526</v>
       </c>
@@ -5287,7 +5296,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" s="8" t="s">
         <v>528</v>
       </c>
@@ -5298,7 +5307,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="261" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" s="8" t="s">
         <v>530</v>
       </c>
@@ -5309,7 +5318,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" s="8" t="s">
         <v>532</v>
       </c>
@@ -5320,7 +5329,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="263" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263" s="8" t="s">
         <v>534</v>
       </c>
@@ -5331,7 +5340,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="264" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" s="8" t="s">
         <v>536</v>
       </c>
@@ -5342,7 +5351,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A265" s="8" t="s">
         <v>538</v>
       </c>
@@ -5353,7 +5362,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="266" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266" s="8" t="s">
         <v>540</v>
       </c>
@@ -5364,7 +5373,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="267" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A267" s="8" t="s">
         <v>542</v>
       </c>
@@ -5375,7 +5384,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="268" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A268" s="8" t="s">
         <v>544</v>
       </c>
@@ -5386,7 +5395,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="269" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A269" s="8" t="s">
         <v>546</v>
       </c>
@@ -5397,7 +5406,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="270" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A270" s="8" t="s">
         <v>548</v>
       </c>
@@ -5408,7 +5417,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="271" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271" s="8" t="s">
         <v>550</v>
       </c>
@@ -5419,7 +5428,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="272" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A272" s="8" t="s">
         <v>552</v>
       </c>
@@ -5430,7 +5439,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="273" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A273" s="8" t="s">
         <v>554</v>
       </c>
@@ -5441,7 +5450,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="274" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A274" s="8" t="s">
         <v>556</v>
       </c>
@@ -5452,7 +5461,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="275" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275" s="8" t="s">
         <v>558</v>
       </c>
@@ -5463,7 +5472,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="276" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276" s="9" t="s">
         <v>560</v>
       </c>
@@ -5474,7 +5483,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="277" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" s="8" t="s">
         <v>562</v>
       </c>
@@ -5485,7 +5494,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="278" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A278" s="8" t="s">
         <v>564</v>
       </c>
@@ -5496,7 +5505,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="279" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A279" s="8" t="s">
         <v>566</v>
       </c>
@@ -5507,7 +5516,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="280" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A280" s="9" t="s">
         <v>568</v>
       </c>
@@ -5518,7 +5527,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="281" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A281" s="8" t="s">
         <v>570</v>
       </c>
@@ -5529,7 +5538,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="282" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A282" s="8" t="s">
         <v>572</v>
       </c>
@@ -5540,7 +5549,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="283" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283" s="9" t="s">
         <v>574</v>
       </c>
@@ -5551,7 +5560,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="284" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A284" s="8" t="s">
         <v>576</v>
       </c>
@@ -5562,7 +5571,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="285" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A285" s="9" t="s">
         <v>578</v>
       </c>
@@ -5573,7 +5582,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="286" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286" s="3" t="s">
         <v>7</v>
       </c>
@@ -5584,7 +5593,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="287" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A287" s="3" t="s">
         <v>4</v>
       </c>
@@ -5595,7 +5604,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="288" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A288" s="3" t="s">
         <v>11</v>
       </c>
@@ -5606,7 +5615,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="289" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A289" s="3" t="s">
         <v>6</v>
       </c>
@@ -5617,7 +5626,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="290" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A290" s="3" t="s">
         <v>9</v>
       </c>
@@ -5628,7 +5637,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="291" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A291" s="3" t="s">
         <v>5</v>
       </c>
@@ -5639,7 +5648,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="292" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A292" s="3" t="s">
         <v>10</v>
       </c>
@@ -5650,7 +5659,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="293" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A293" s="3" t="s">
         <v>8</v>
       </c>
@@ -5661,7 +5670,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="294" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A294" s="3" t="s">
         <v>587</v>
       </c>
@@ -5672,7 +5681,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="295" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A295" s="2" t="s">
         <v>589</v>
       </c>
@@ -5683,7 +5692,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="296" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A296" s="2" t="s">
         <v>591</v>
       </c>
@@ -5694,7 +5703,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="297" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A297" s="2" t="s">
         <v>593</v>
       </c>
@@ -5705,7 +5714,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="298" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A298" s="2" t="s">
         <v>574</v>
       </c>
@@ -5716,7 +5725,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="299" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A299" s="3" t="s">
         <v>576</v>
       </c>
@@ -5727,7 +5736,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="300" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A300" s="2" t="s">
         <v>578</v>
       </c>
@@ -5738,7 +5747,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="301" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A301" s="3" t="s">
         <v>595</v>
       </c>
@@ -5749,7 +5758,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="302" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A302" s="3" t="s">
         <v>596</v>
       </c>
@@ -5760,7 +5769,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="303" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A303" s="3" t="s">
         <v>597</v>
       </c>
@@ -5771,7 +5780,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="304" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A304" s="3" t="s">
         <v>598</v>
       </c>
@@ -5782,7 +5791,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="305" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A305" s="3" t="s">
         <v>599</v>
       </c>
@@ -5793,7 +5802,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="306" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A306" s="3" t="s">
         <v>600</v>
       </c>
@@ -5804,7 +5813,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="307" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A307" s="3" t="s">
         <v>601</v>
       </c>
@@ -5815,7 +5824,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="308" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A308" s="3" t="s">
         <v>602</v>
       </c>
@@ -5826,7 +5835,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="309" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A309" s="3" t="s">
         <v>603</v>
       </c>
@@ -5837,7 +5846,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="310" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A310" s="3" t="s">
         <v>604</v>
       </c>
@@ -5848,7 +5857,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="311" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A311" s="3" t="s">
         <v>605</v>
       </c>
@@ -5859,7 +5868,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="312" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A312" s="3" t="s">
         <v>607</v>
       </c>
@@ -5870,7 +5879,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="313" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A313" s="3" t="s">
         <v>608</v>
       </c>
@@ -5881,7 +5890,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="314" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A314" s="3" t="s">
         <v>609</v>
       </c>
@@ -5892,7 +5901,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="315" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A315" s="3" t="s">
         <v>611</v>
       </c>
@@ -5903,7 +5912,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="316" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A316" s="3" t="s">
         <v>613</v>
       </c>
@@ -5914,7 +5923,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="317" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A317" s="3" t="s">
         <v>614</v>
       </c>
@@ -5925,7 +5934,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="318" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A318" s="3" t="s">
         <v>615</v>
       </c>
@@ -5936,7 +5945,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="319" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A319" s="3" t="s">
         <v>616</v>
       </c>
@@ -5947,7 +5956,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="320" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A320" s="3" t="s">
         <v>617</v>
       </c>
@@ -5958,7 +5967,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="321" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A321" s="3" t="s">
         <v>618</v>
       </c>
@@ -5969,7 +5978,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="322" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A322" s="3" t="s">
         <v>619</v>
       </c>
@@ -5980,7 +5989,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="323" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A323" s="3" t="s">
         <v>620</v>
       </c>
@@ -5991,7 +6000,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="324" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A324" s="3" t="s">
         <v>621</v>
       </c>
@@ -6002,7 +6011,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="325" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A325" s="3" t="s">
         <v>623</v>
       </c>
@@ -6013,7 +6022,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="326" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A326" s="11" t="s">
         <v>620</v>
       </c>
@@ -6024,7 +6033,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="327" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A327" s="11" t="s">
         <v>621</v>
       </c>
@@ -6035,7 +6044,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="328" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A328" s="11" t="s">
         <v>623</v>
       </c>
@@ -6046,7 +6055,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="329" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A329" s="10" t="s">
         <v>445</v>
       </c>
@@ -6057,7 +6066,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="330" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A330" s="10" t="s">
         <v>627</v>
       </c>
@@ -6068,7 +6077,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="331" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A331" s="3" t="s">
         <v>12</v>
       </c>
@@ -6079,7 +6088,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="332" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A332" s="3" t="s">
         <v>631</v>
       </c>
@@ -6090,7 +6099,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="333" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A333" s="3" t="s">
         <v>633</v>
       </c>
@@ -6101,7 +6110,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="334" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A334" s="3" t="s">
         <v>635</v>
       </c>
@@ -6112,7 +6121,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="335" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A335" s="3" t="s">
         <v>637</v>
       </c>
@@ -6123,7 +6132,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="336" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A336" s="3" t="s">
         <v>639</v>
       </c>
@@ -6134,7 +6143,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="337" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A337" s="3" t="s">
         <v>586</v>
       </c>
@@ -6145,7 +6154,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="338" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A338" s="3" t="s">
         <v>583</v>
       </c>
@@ -6156,7 +6165,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="339" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A339" s="3" t="s">
         <v>581</v>
       </c>
@@ -6167,7 +6176,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="340" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A340" s="3" t="s">
         <v>13</v>
       </c>
@@ -6178,7 +6187,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="341" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A341" s="3" t="s">
         <v>585</v>
       </c>
@@ -6189,7 +6198,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="342" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A342" s="3" t="s">
         <v>584</v>
       </c>
@@ -6200,7 +6209,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="343" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A343" s="3" t="s">
         <v>582</v>
       </c>
@@ -6211,7 +6220,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="344" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A344" s="3" t="s">
         <v>648</v>
       </c>
@@ -6222,7 +6231,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="345" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A345" s="3" t="s">
         <v>650</v>
       </c>
@@ -6233,7 +6242,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="346" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A346" s="3" t="s">
         <v>652</v>
       </c>
@@ -6244,7 +6253,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="347" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
         <v>654</v>
       </c>
@@ -6252,6 +6261,28 @@
         <v>630</v>
       </c>
       <c r="C347" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="348" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A348" s="12" t="s">
+        <v>655</v>
+      </c>
+      <c r="B348" s="3" t="s">
+        <v>656</v>
+      </c>
+      <c r="C348" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="349" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A349" t="s">
+        <v>657</v>
+      </c>
+      <c r="B349" t="s">
+        <v>658</v>
+      </c>
+      <c r="C349" s="6" t="s">
         <v>3</v>
       </c>
     </row>
@@ -6935,7 +6966,9 @@
     <hyperlink ref="B344" r:id="rId676" display="https://www.addact.net/hire-expert/umbraco-developer" xr:uid="{FCDDBDCE-1843-4317-94E4-1B70EB9DBF04}"/>
     <hyperlink ref="B345" r:id="rId677" display="https://www.addact.net/hire-expert/strapi-developer" xr:uid="{E4D49E07-6A2F-4A09-AC25-A47B8CB158B6}"/>
     <hyperlink ref="B346" r:id="rId678" display="https://www.addact.net/hire-experts/kentico-developer" xr:uid="{0DE63966-9454-4E7F-9874-4FB7691962D7}"/>
+    <hyperlink ref="B348" r:id="rId679" display="https://www.addact.net/contact-us" xr:uid="{8D2B2D29-8851-40E3-8574-33F6447C6FD5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId680"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated redirects rule for ui-ux-design-services page
</commit_message>
<xml_diff>
--- a/addact/public/redirects.xlsx
+++ b/addact/public/redirects.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Addact-Revamp\addact\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\Addact-Revamp\addact\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6EE1969-9EDA-46C7-BBCD-4FBAF73A9D5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23360FDC-63C2-4642-8494-C75A5AA5C8AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{5F6600C6-C08A-47D2-B3C8-F7A43562057B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5F6600C6-C08A-47D2-B3C8-F7A43562057B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="659">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1049" uniqueCount="661">
   <si>
     <t>source</t>
   </si>
@@ -2002,6 +2002,12 @@
   </si>
   <si>
     <t>/project-cost-estimators</t>
+  </si>
+  <si>
+    <t>/digital-marketing/ui-ux-design-services</t>
+  </si>
+  <si>
+    <t>/development-design/ui-ux-design-services</t>
   </si>
 </sst>
 </file>
@@ -2439,7 +2445,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C59FA00F-2D8F-4BC7-B234-D60C0BA408AE}">
-  <dimension ref="A1:C349"/>
+  <dimension ref="A1:C350"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="107.42578125" customWidth="1"/>
@@ -6284,6 +6290,17 @@
       </c>
       <c r="C349" s="6" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="350" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A350" t="s">
+        <v>660</v>
+      </c>
+      <c r="B350" t="s">
+        <v>659</v>
+      </c>
+      <c r="C350" s="7" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added redirection for UIUX page
</commit_message>
<xml_diff>
--- a/addact/public/redirects.xlsx
+++ b/addact/public/redirects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\Addact-Revamp\addact\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23360FDC-63C2-4642-8494-C75A5AA5C8AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68911555-E93B-4F3F-B2E6-EE9E61374E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5F6600C6-C08A-47D2-B3C8-F7A43562057B}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1049" uniqueCount="661">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1050" uniqueCount="661">
   <si>
     <t>source</t>
   </si>
@@ -6299,8 +6299,8 @@
       <c r="B350" t="s">
         <v>659</v>
       </c>
-      <c r="C350" s="7" t="b">
-        <v>1</v>
+      <c r="C350" s="6" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: redirect rule for the sitecore/platform-upgrade route
</commit_message>
<xml_diff>
--- a/addact/public/redirects.xlsx
+++ b/addact/public/redirects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\Addact-Revamp\addact\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{729BB614-7C2A-4B9E-B1DD-040D8670AF85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7461A1-E607-442F-A1E3-A276190C5BC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5F6600C6-C08A-47D2-B3C8-F7A43562057B}"/>
   </bookViews>
@@ -6124,7 +6124,7 @@
         <v>12</v>
       </c>
       <c r="B331" s="3" t="s">
-        <v>630</v>
+        <v>661</v>
       </c>
       <c r="C331" s="6" t="s">
         <v>3</v>
@@ -6135,7 +6135,7 @@
         <v>631</v>
       </c>
       <c r="B332" s="3" t="s">
-        <v>632</v>
+        <v>662</v>
       </c>
       <c r="C332" s="6" t="s">
         <v>3</v>
@@ -6146,7 +6146,7 @@
         <v>633</v>
       </c>
       <c r="B333" s="3" t="s">
-        <v>634</v>
+        <v>663</v>
       </c>
       <c r="C333" s="6" t="s">
         <v>3</v>
@@ -6157,7 +6157,7 @@
         <v>635</v>
       </c>
       <c r="B334" s="3" t="s">
-        <v>636</v>
+        <v>664</v>
       </c>
       <c r="C334" s="6" t="s">
         <v>3</v>
@@ -6168,7 +6168,7 @@
         <v>637</v>
       </c>
       <c r="B335" s="3" t="s">
-        <v>638</v>
+        <v>665</v>
       </c>
       <c r="C335" s="6" t="s">
         <v>3</v>
@@ -6179,7 +6179,7 @@
         <v>639</v>
       </c>
       <c r="B336" s="3" t="s">
-        <v>640</v>
+        <v>666</v>
       </c>
       <c r="C336" s="6" t="s">
         <v>3</v>
@@ -6190,7 +6190,7 @@
         <v>586</v>
       </c>
       <c r="B337" s="3" t="s">
-        <v>641</v>
+        <v>667</v>
       </c>
       <c r="C337" s="6" t="s">
         <v>3</v>
@@ -6201,7 +6201,7 @@
         <v>583</v>
       </c>
       <c r="B338" s="3" t="s">
-        <v>642</v>
+        <v>668</v>
       </c>
       <c r="C338" s="6" t="s">
         <v>3</v>
@@ -6212,7 +6212,7 @@
         <v>581</v>
       </c>
       <c r="B339" s="3" t="s">
-        <v>643</v>
+        <v>669</v>
       </c>
       <c r="C339" s="6" t="s">
         <v>3</v>
@@ -6223,7 +6223,7 @@
         <v>13</v>
       </c>
       <c r="B340" s="3" t="s">
-        <v>644</v>
+        <v>670</v>
       </c>
       <c r="C340" s="6" t="s">
         <v>3</v>
@@ -6234,7 +6234,7 @@
         <v>585</v>
       </c>
       <c r="B341" s="3" t="s">
-        <v>645</v>
+        <v>671</v>
       </c>
       <c r="C341" s="6" t="s">
         <v>3</v>
@@ -6245,7 +6245,7 @@
         <v>584</v>
       </c>
       <c r="B342" s="3" t="s">
-        <v>646</v>
+        <v>672</v>
       </c>
       <c r="C342" s="6" t="s">
         <v>3</v>
@@ -6300,7 +6300,7 @@
         <v>654</v>
       </c>
       <c r="B347" t="s">
-        <v>630</v>
+        <v>661</v>
       </c>
       <c r="C347" s="6" t="s">
         <v>3</v>
@@ -6462,7 +6462,7 @@
     </row>
     <row r="362" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>672</v>
+        <v>646</v>
       </c>
       <c r="B362" t="s">
         <v>672</v>

</xml_diff>

<commit_message>
Redirection rule added for uiux services page
</commit_message>
<xml_diff>
--- a/addact/public/redirects.xlsx
+++ b/addact/public/redirects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\Addact-Revamp\addact\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7461A1-E607-442F-A1E3-A276190C5BC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86733BF6-C54E-4B61-9098-45CFEE826001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5F6600C6-C08A-47D2-B3C8-F7A43562057B}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1086" uniqueCount="673">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="674">
   <si>
     <t>source</t>
   </si>
@@ -2044,6 +2044,9 @@
   </si>
   <si>
     <t>/development-services/cms-development/sitecore/platform-upgrade</t>
+  </si>
+  <si>
+    <t>/development-services/ui-ux-design-services</t>
   </si>
 </sst>
 </file>
@@ -2481,7 +2484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C59FA00F-2D8F-4BC7-B234-D60C0BA408AE}">
-  <dimension ref="A1:C362"/>
+  <dimension ref="A1:C363"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="107.42578125" customWidth="1"/>
@@ -6468,6 +6471,17 @@
         <v>672</v>
       </c>
       <c r="C362" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="363" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A363" t="s">
+        <v>673</v>
+      </c>
+      <c r="B363" t="s">
+        <v>659</v>
+      </c>
+      <c r="C363" s="6" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>